<commit_message>
fix(report): address all P2 exit review findings
Signed-off-by: bora <bora@post.cz>
</commit_message>
<xml_diff>
--- a/packages/kotlin/ttr-report-cli/src/test/resources/worlds/reports/expected.xlsx
+++ b/packages/kotlin/ttr-report-cli/src/test/resources/worlds/reports/expected.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>{{title}}</t>
   </si>
@@ -48,35 +48,16 @@
     <t>Parts &amp; &lt;kits&gt;</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>001.50</t>
-  </si>
-  <si>
     <t>Service</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>20.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.###############"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <sz val="11.0"/>
@@ -116,10 +97,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true">
+      <alignment wrapText="true"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -137,12 +133,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="2">
+      <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" s="0" t="s">
         <v>9</v>
       </c>
     </row>
@@ -163,38 +159,38 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15.0" customHeight="true">
-      <c r="A4" t="s" s="0">
+    <row r="4">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="4" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>12</v>
+      <c r="B5" s="4" t="n">
+        <v>8.0</v>
       </c>
-      <c r="D4" s="0" t="s">
-        <v>13</v>
+      <c r="C5" s="5" t="n">
+        <v>7.0</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>14</v>
+      <c r="D5" s="6" t="n">
+        <v>1.0</v>
       </c>
-    </row>
-    <row r="5" ht="15.0" customHeight="true">
-      <c r="A5" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="0" t="s">
-        <v>18</v>
+      <c r="E5" s="7" t="n">
+        <v>20.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>